<commit_message>
restage the fixture: contract category labels, and a narrative that fits this deal
Two changes reach the published set. The T-12 category labels now match the
production skill's contract character-exact (General and Administrative, not G&A;
Gain / (Loss) to Lease with its spaces) - they are a join key, and a drifted one
matches nothing while erroring nowhere.

And the comp-set narrative is derived from the fixture's own swap instead of a
template. It previously said one community was "replaced" when one was added and
none removed, and called the newcomer "newer" when it is older than every
community in set A. Both now come from the facts.
</commit_message>
<xml_diff>
--- a/public/downloads/underwriting-demo/sample-model-ready-outputs.xlsx
+++ b/public/downloads/underwriting-demo/sample-model-ready-outputs.xlsx
@@ -3158,7 +3158,7 @@
       </c>
       <c r="B86" s="6" t="inlineStr">
         <is>
-          <t>Gain/(Loss) to Lease</t>
+          <t>Gain / (Loss) to Lease</t>
         </is>
       </c>
       <c r="C86" s="6" t="inlineStr">
@@ -3168,7 +3168,7 @@
       </c>
       <c r="D86" s="7" t="inlineStr">
         <is>
-          <t>Gain/(Loss) to Lease — trailing-twelve total, and trailing-three annualized beside it.</t>
+          <t>Gain / (Loss) to Lease — trailing-twelve total, and trailing-three annualized beside it.</t>
         </is>
       </c>
       <c r="E86" s="6" t="inlineStr">
@@ -3541,7 +3541,7 @@
       </c>
       <c r="B97" s="6" t="inlineStr">
         <is>
-          <t>G&amp;A</t>
+          <t>General and Administrative</t>
         </is>
       </c>
       <c r="C97" s="6" t="inlineStr">
@@ -3551,7 +3551,7 @@
       </c>
       <c r="D97" s="7" t="inlineStr">
         <is>
-          <t>G&amp;A — trailing-twelve total, trailing-three annualized, and per unit.</t>
+          <t>General and Administrative — trailing-twelve total, trailing-three annualized, and per unit.</t>
         </is>
       </c>
       <c r="E97" s="6" t="inlineStr">

</xml_diff>